<commit_message>
feat: implement admin and student dashboard pages with grid mode visualization for database management
</commit_message>
<xml_diff>
--- a/TMSL - B.Tech- (CSE,IT, CSE-AIML,CSBS,CSDS ,CSCS,ECE,ECS,CSE-IOT,EE,EIE,ME,CE,FT) -MASTER DATABASE FORMAT- 2027 pass out batch (1).xlsx
+++ b/TMSL - B.Tech- (CSE,IT, CSE-AIML,CSBS,CSDS ,CSCS,ECE,ECS,CSE-IOT,EE,EIE,ME,CE,FT) -MASTER DATABASE FORMAT- 2027 pass out batch (1).xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\TMSL AIML Master Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E425D40-82AF-4E66-9F7F-7BD6A2D015E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -314,9 +315,6 @@
     <t>CSE/IT/ CSE- AIML / CSBS / CSDS / CSCS/ ECE/EE/EIE/ME/CE/FT</t>
   </si>
   <si>
-    <t xml:space="preserve">  UPLOAD LINK OF UPDATED FORMAL PHOTO IN PDF FORMAT ( Mamdatory Field)</t>
-  </si>
-  <si>
     <t xml:space="preserve">DIPLOMA DETAILS ( IF APPLICABLE) </t>
   </si>
   <si>
@@ -335,12 +333,15 @@
   </si>
   <si>
     <t>2023-2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  UPLOAD LINK OF UPDATED FORMAL PHOTO IN PDF FORMAT ( Mandatory Field)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="0.00;[Red]0.00"/>
@@ -1197,7 +1198,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1257,10 +1258,15 @@
     <xf numFmtId="0" fontId="19" fillId="37" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1316,15 +1322,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="43" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1392,9 +1389,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1432,9 +1429,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1469,7 +1466,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1504,7 +1501,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1677,7 +1674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CH15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1761,110 +1758,110 @@
   <sheetData>
     <row r="1" spans="1:86" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:86" s="2" customFormat="1" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
       <c r="P2" s="22"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="25" t="s">
+      <c r="Q2" s="22"/>
+      <c r="R2" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="26"/>
-      <c r="Y2" s="26"/>
-      <c r="Z2" s="26"/>
-      <c r="AA2" s="27"/>
-      <c r="AB2" s="38" t="s">
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="27"/>
+      <c r="Y2" s="27"/>
+      <c r="Z2" s="27"/>
+      <c r="AA2" s="28"/>
+      <c r="AB2" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="AC2" s="39"/>
-      <c r="AD2" s="39"/>
-      <c r="AE2" s="39"/>
-      <c r="AF2" s="39"/>
-      <c r="AG2" s="39"/>
-      <c r="AH2" s="39"/>
-      <c r="AI2" s="39"/>
-      <c r="AJ2" s="39"/>
-      <c r="AK2" s="40"/>
-      <c r="AL2" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM2" s="42"/>
-      <c r="AN2" s="42"/>
-      <c r="AO2" s="42"/>
-      <c r="AP2" s="42"/>
-      <c r="AQ2" s="42"/>
-      <c r="AR2" s="43"/>
-      <c r="AS2" s="33" t="s">
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="41"/>
+      <c r="AL2" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM2" s="43"/>
+      <c r="AN2" s="43"/>
+      <c r="AO2" s="43"/>
+      <c r="AP2" s="43"/>
+      <c r="AQ2" s="43"/>
+      <c r="AR2" s="44"/>
+      <c r="AS2" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="AT2" s="33"/>
-      <c r="AU2" s="33"/>
-      <c r="AV2" s="33"/>
-      <c r="AW2" s="33"/>
-      <c r="AX2" s="33"/>
-      <c r="AY2" s="33"/>
-      <c r="AZ2" s="33"/>
-      <c r="BA2" s="33"/>
-      <c r="BB2" s="33"/>
-      <c r="BC2" s="33"/>
-      <c r="BD2" s="33"/>
-      <c r="BE2" s="33"/>
-      <c r="BF2" s="33"/>
-      <c r="BG2" s="33"/>
-      <c r="BH2" s="34" t="s">
+      <c r="AT2" s="34"/>
+      <c r="AU2" s="34"/>
+      <c r="AV2" s="34"/>
+      <c r="AW2" s="34"/>
+      <c r="AX2" s="34"/>
+      <c r="AY2" s="34"/>
+      <c r="AZ2" s="34"/>
+      <c r="BA2" s="34"/>
+      <c r="BB2" s="34"/>
+      <c r="BC2" s="34"/>
+      <c r="BD2" s="34"/>
+      <c r="BE2" s="34"/>
+      <c r="BF2" s="34"/>
+      <c r="BG2" s="34"/>
+      <c r="BH2" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="BI2" s="34"/>
-      <c r="BJ2" s="34"/>
-      <c r="BK2" s="34"/>
-      <c r="BL2" s="34"/>
-      <c r="BM2" s="34"/>
-      <c r="BN2" s="34"/>
-      <c r="BO2" s="35" t="s">
+      <c r="BI2" s="35"/>
+      <c r="BJ2" s="35"/>
+      <c r="BK2" s="35"/>
+      <c r="BL2" s="35"/>
+      <c r="BM2" s="35"/>
+      <c r="BN2" s="35"/>
+      <c r="BO2" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="BP2" s="35"/>
-      <c r="BQ2" s="35"/>
-      <c r="BR2" s="35"/>
-      <c r="BS2" s="35"/>
-      <c r="BT2" s="35"/>
-      <c r="BU2" s="36" t="s">
+      <c r="BP2" s="36"/>
+      <c r="BQ2" s="36"/>
+      <c r="BR2" s="36"/>
+      <c r="BS2" s="36"/>
+      <c r="BT2" s="36"/>
+      <c r="BU2" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="BV2" s="36"/>
-      <c r="BW2" s="36"/>
-      <c r="BX2" s="36"/>
-      <c r="BY2" s="36"/>
-      <c r="BZ2" s="37"/>
-      <c r="CA2" s="30" t="s">
+      <c r="BV2" s="37"/>
+      <c r="BW2" s="37"/>
+      <c r="BX2" s="37"/>
+      <c r="BY2" s="37"/>
+      <c r="BZ2" s="38"/>
+      <c r="CA2" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="CB2" s="31"/>
-      <c r="CC2" s="31"/>
-      <c r="CD2" s="31"/>
-      <c r="CE2" s="31"/>
-      <c r="CF2" s="31"/>
-      <c r="CG2" s="31"/>
-      <c r="CH2" s="32"/>
+      <c r="CB2" s="32"/>
+      <c r="CC2" s="32"/>
+      <c r="CD2" s="32"/>
+      <c r="CE2" s="32"/>
+      <c r="CF2" s="32"/>
+      <c r="CG2" s="32"/>
+      <c r="CH2" s="33"/>
     </row>
     <row r="3" spans="1:86" s="5" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
@@ -1886,7 +1883,7 @@
         <v>3</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>29</v>
@@ -1912,11 +1909,11 @@
       <c r="O3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="44" t="s">
+      <c r="P3" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q3" s="23" t="s">
         <v>100</v>
-      </c>
-      <c r="Q3" s="44" t="s">
-        <v>101</v>
       </c>
       <c r="R3" s="12" t="s">
         <v>74</v>
@@ -2131,7 +2128,7 @@
     </row>
     <row r="5" spans="1:86" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>79</v>
@@ -2148,10 +2145,10 @@
       <c r="M5" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="N5" s="45" t="s">
-        <v>102</v>
-      </c>
-      <c r="O5" s="46" t="s">
+      <c r="N5" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="O5" s="25" t="s">
         <v>40</v>
       </c>
       <c r="P5" s="8"/>
@@ -2199,7 +2196,7 @@
         <v>96</v>
       </c>
       <c r="AW5" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="BD5" s="6" t="s">
         <v>80</v>
@@ -2264,8 +2261,6 @@
     <row r="14" spans="1:86" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:86" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O15" s="4"/>
-      <c r="P15" s="24"/>
-      <c r="Q15" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2280,7 +2275,7 @@
     <mergeCell ref="AL2:AR2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O5" r:id="rId1"/>
+    <hyperlink ref="O5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
@@ -2288,7 +2283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>